<commit_message>
Quartz sync: Sep 30, 2025, 9:40 PM
</commit_message>
<xml_diff>
--- a/content/Notes/Biology/Labs/Lab 03/Book1.xlsx
+++ b/content/Notes/Biology/Labs/Lab 03/Book1.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10913"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10921"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gassandrid/VAULT/Notes/Biology/Labs/Lab 03/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2FF7CD0-D0AD-D543-842D-A74B475D38CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEB82866-6D43-D74D-89B1-2648AF910989}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="60" yWindow="740" windowWidth="34440" windowHeight="21540" xr2:uid="{E530C7BC-18CB-1A4A-8AEB-68DCBA488E9C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Trial</t>
   </si>
@@ -69,87 +69,6 @@
   </si>
   <si>
     <t>Test</t>
-  </si>
-  <si>
-    <t>ican Vidallowers</t>
-  </si>
-  <si>
-    <t>Condusion</t>
-  </si>
-  <si>
-    <t>-What do your results mean?</t>
-  </si>
-  <si>
-    <t>Unpack Interpret your data</t>
-  </si>
-  <si>
-    <t>Leg p-vale =0.0041 &lt;0.05</t>
-  </si>
-  <si>
-    <t>this means there is a stat sig dity</t>
-  </si>
-  <si>
-    <t>→ Discuss your hypothesis in the context of your +-test</t>
-  </si>
-  <si>
-    <t>Does your data support your hypo?</t>
-  </si>
-  <si>
-    <t>Inconcusive? How do you know?</t>
-  </si>
-  <si>
-    <t>→ Were there confanding variables</t>
-  </si>
-  <si>
-    <t>that decrease your confidence</t>
-  </si>
-  <si>
-    <t>in your claims /evidence?</t>
-  </si>
-  <si>
-    <t>→ Haw would ya change the experiment</t>
-  </si>
-  <si>
-    <t>in the future?</t>
-  </si>
-  <si>
-    <t>Results</t>
-  </si>
-  <si>
-    <t>→ Just the numbers!</t>
-  </si>
-  <si>
-    <t>→ What stat test were used leg, SDs, t. test →p-valu → about observations that provide context to your resuts leg, trial 2 had a small sample? compared to the others</t>
-  </si>
-  <si>
-    <t>- Contarinotion?</t>
-  </si>
-  <si>
-    <t>﻿Heat exposure</t>
-  </si>
-  <si>
-    <t>﻿﻿Slide movement</t>
-  </si>
-  <si>
-    <t>﻿﻿Distance of drops and Diffusion of solution over time?</t>
-  </si>
-  <si>
-    <t>﻿﻿Experimental error</t>
-  </si>
-  <si>
-    <t>THuran Eror?]</t>
-  </si>
-  <si>
-    <t>﻿﻿What was hard to Control for?</t>
-  </si>
-  <si>
-    <t>Buc</t>
-  </si>
-  <si>
-    <t>of Norti</t>
-  </si>
-  <si>
-    <t>America</t>
   </si>
 </sst>
 </file>
@@ -233,6 +152,997 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$I$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Average</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:errBars>
+            <c:errBarType val="both"/>
+            <c:errValType val="cust"/>
+            <c:noEndCap val="0"/>
+            <c:plus>
+              <c:numRef>
+                <c:f>Sheet1!$J$2:$J$3</c:f>
+                <c:numCache>
+                  <c:formatCode>General</c:formatCode>
+                  <c:ptCount val="2"/>
+                  <c:pt idx="0">
+                    <c:v>0.30034703199697804</c:v>
+                  </c:pt>
+                  <c:pt idx="1">
+                    <c:v>0</c:v>
+                  </c:pt>
+                </c:numCache>
+              </c:numRef>
+            </c:plus>
+            <c:minus>
+              <c:numLit>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+              </c:numLit>
+            </c:minus>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:round/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:errBars>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$H$2:$H$3</c:f>
+              <c:strCache>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>Control</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Test</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$I$2:$I$3</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>0.37126984126000001</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-94B3-9C46-9623-7837BF300AF4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="1650827936"/>
+        <c:axId val="298424288"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1650827936"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Solution</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> Type</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="298424288"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="298424288"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Average</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> Proportion of Paramecium</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1650827936"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>8842</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>83273</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>312677</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>13182</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{30C2886C-E8F7-9CB7-8171-DF258B13794C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -815,146 +1725,92 @@
       </c>
     </row>
     <row r="17" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I17" s="3">
-        <v>3</v>
-      </c>
+      <c r="I17" s="3"/>
     </row>
     <row r="18" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I18" s="3" t="s">
-        <v>11</v>
-      </c>
+      <c r="I18" s="3"/>
     </row>
     <row r="19" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I19" s="3" t="s">
-        <v>12</v>
-      </c>
+      <c r="I19" s="3"/>
     </row>
     <row r="20" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I20" s="3" t="s">
-        <v>13</v>
-      </c>
+      <c r="I20" s="3"/>
     </row>
     <row r="21" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I21" s="3" t="s">
-        <v>14</v>
-      </c>
+      <c r="I21" s="3"/>
     </row>
     <row r="22" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I22" s="3" t="s">
-        <v>15</v>
-      </c>
+      <c r="I22" s="3"/>
     </row>
     <row r="23" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I23" s="3" t="s">
-        <v>16</v>
-      </c>
+      <c r="I23" s="3"/>
     </row>
     <row r="24" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I24" s="3" t="s">
-        <v>17</v>
-      </c>
+      <c r="I24" s="3"/>
     </row>
     <row r="25" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I25" s="3" t="s">
-        <v>18</v>
-      </c>
+      <c r="I25" s="3"/>
     </row>
     <row r="26" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I26" s="3" t="s">
-        <v>19</v>
-      </c>
+      <c r="I26" s="3"/>
     </row>
     <row r="27" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I27" s="3" t="s">
-        <v>20</v>
-      </c>
+      <c r="I27" s="3"/>
     </row>
     <row r="28" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I28" s="3" t="s">
-        <v>21</v>
-      </c>
+      <c r="I28" s="3"/>
     </row>
     <row r="29" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I29" s="3" t="s">
-        <v>22</v>
-      </c>
+      <c r="I29" s="3"/>
     </row>
     <row r="30" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I30" s="3" t="s">
-        <v>23</v>
-      </c>
+      <c r="I30" s="3"/>
     </row>
     <row r="31" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I31" s="3" t="s">
-        <v>24</v>
-      </c>
+      <c r="I31" s="3"/>
     </row>
     <row r="32" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I32" s="3" t="s">
-        <v>25</v>
-      </c>
+      <c r="I32" s="3"/>
     </row>
     <row r="33" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I33" s="3" t="s">
-        <v>26</v>
-      </c>
+      <c r="I33" s="3"/>
     </row>
     <row r="34" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I34" s="3" t="s">
-        <v>27</v>
-      </c>
+      <c r="I34" s="3"/>
     </row>
     <row r="35" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I35" s="3" t="s">
-        <v>28</v>
-      </c>
+      <c r="I35" s="3"/>
     </row>
     <row r="37" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I37" s="3" t="s">
-        <v>29</v>
-      </c>
+      <c r="I37" s="3"/>
     </row>
     <row r="38" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I38" s="3" t="s">
-        <v>30</v>
-      </c>
+      <c r="I38" s="3"/>
     </row>
     <row r="39" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I39" s="3" t="s">
-        <v>31</v>
-      </c>
+      <c r="I39" s="3"/>
     </row>
     <row r="40" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I40" s="3" t="s">
-        <v>32</v>
-      </c>
+      <c r="I40" s="3"/>
     </row>
     <row r="41" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I41" s="3" t="s">
-        <v>33</v>
-      </c>
+      <c r="I41" s="3"/>
     </row>
     <row r="42" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I42" s="3" t="s">
-        <v>34</v>
-      </c>
+      <c r="I42" s="3"/>
     </row>
     <row r="44" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I44" s="3" t="s">
-        <v>35</v>
-      </c>
+      <c r="I44" s="3"/>
     </row>
     <row r="45" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I45" s="3" t="s">
-        <v>36</v>
-      </c>
+      <c r="I45" s="3"/>
     </row>
     <row r="46" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I46" s="3" t="s">
-        <v>37</v>
-      </c>
+      <c r="I46" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>